<commit_message>
Sync all local changes including extractors
</commit_message>
<xml_diff>
--- a/Uyumsoft_Aktarim_Taslagi.xlsx
+++ b/Uyumsoft_Aktarim_Taslagi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,52 +471,312 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7.07.2026</t>
+          <t>15.08.2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11111111111</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0213.217</t>
+          <t>8100.003</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NFC Silver Kart</t>
+          <t>Plastik Kart Tasarımı</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>10,00</t>
+          <t>2,0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>40,00</t>
+          <t>15,75</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>400,00</t>
+          <t>31,50</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>400,00</t>
+          <t>6.350,75</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>80,00</t>
+          <t>1.143,14</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>480,00</t>
+          <t>6.858,81</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>15.08.2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>9001.452</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Kargo ve Lojistik Bedeli</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>10,0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>275,50</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2.755,00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>6.350,75</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1.143,14</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>6.858,81</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>15.08.2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3300.517</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NFC Encoder Cihazı</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>5,0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>600,00</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3.000,00</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>6.350,75</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1.143,14</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>6.858,81</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>15.08.2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7700.224</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Etiket Baskı Hizmeti</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>5,0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>15,25</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>76,25</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>6.350,75</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1.143,14</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>6.858,81</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>15.08.2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>6500.332</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sistem Kurulum Danışmanlığı</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4,0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>48,00</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>6.350,75</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>1.143,14</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>6.858,81</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>15.08.2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1250.811</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Demo Kart Paketi</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>8,0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>55,00</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>440,00</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>6.350,75</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1.143,14</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>6.858,81</t>
         </is>
       </c>
     </row>

</xml_diff>